<commit_message>
finance: mark Supabase/Resend/OpenRouter as FREE per founder, rebuild handbooks
- Supabase FREE (not Pro 5) — saves NGN39,675/mo — operating lean now NGN32,990 expected NGN68,715
- Resend FREE 3k/100d + OpenRouter FREE tier verified — note 100/day spike risk
- Beta testers upgraded to PRO — model 50 beta PRO users as NGN37k/mo cost center
- Rebuilt Beta Handbook PDF 30,242 bytes + full Financial Handbook PDF 84,809 bytes with cover, TOC, page numbers, beta costing
- Updated Excel operating budget to reflect FREE tiers (changeable inputs)

Co-authored-by: Philip <tobi@jobiest.ai>
</commit_message>
<xml_diff>
--- a/ai-career-agent-coding-agent/ai-career-agent-coding-agent/finance/Jobiest-Financial-Model.xlsx
+++ b/ai-career-agent-coding-agent/ai-career-agent-coding-agent/finance/Jobiest-Financial-Model.xlsx
@@ -571,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -597,14 +597,14 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Monthly NGN</t>
+          <t>Monthly NGN (×1587)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Vercel Pro</t>
+          <t>Vercel Pro (required for commercial use)</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -625,11 +625,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Supabase Pro</t>
+          <t>Supabase FREE (founder confirmed)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
@@ -646,11 +646,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AI GPT-4o (5M in +1M out)</t>
+          <t>Resend FREE (3k/mo 100/day)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>22.5</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
         <v>1</v>
@@ -667,16 +667,64 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Total USD</t>
-        </is>
+          <t>OpenRouter AI — GPT-4o 5M in +1M out</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
       </c>
       <c r="D5">
-        <f>SUM(D2:D4)</f>
+        <f>B5*C5</f>
         <v/>
       </c>
       <c r="E5">
-        <f>SUM(E2:E4)</f>
-        <v/>
+        <f>D5*1587</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Domain renewal (annual/12)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <f>B6*C6</f>
+        <v/>
+      </c>
+      <c r="E6" t="n">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TOTAL (100 users, GPT-4o)</t>
+        </is>
+      </c>
+      <c r="D7">
+        <f>SUM(D2:D6)</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>SUM(E2:E5)+E6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Supabase FREE saves $25/mo (NGN39,675) — beta cost NGN68,715 not 133k. Beta PRO testers (50 users) ≈ NGN37k/mo AI+hosting as cost center.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>